<commit_message>
feat : ajout d'une autre serie fonctionne -> au cas où la nouvelle série comprend les dates communes -> celles de la nouvelle série sont prises en compte
</commit_message>
<xml_diff>
--- a/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
+++ b/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\px20umf\Documents\github\PlotThoseLines\docs\jdt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C1F4682-41C6-400C-BEB4-93B12D8EF734}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20A08822-01BB-4CF1-A377-F52ADE7891B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1380" yWindow="2865" windowWidth="21600" windowHeight="11745" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="31590" yWindow="1740" windowWidth="21600" windowHeight="11745" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Journal de travail'!$A$6:$G$6</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -42,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="77">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -234,6 +233,45 @@
   </si>
   <si>
     <t xml:space="preserve">Documentation jdt et màj sur github project </t>
+  </si>
+  <si>
+    <t>Explication de quelques nuances du projet par le chef de projet</t>
+  </si>
+  <si>
+    <t>Je constate qu'il reste plus beaucoup de temps pour le projet, il faudra avancer plus, et eventuellement abandonner certains aspects du projet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mise en place de menu latéral permetant de masquer ou d'afficher les graphiques ajoutés </t>
+  </si>
+  <si>
+    <t>Le tableau affiche le nom du graphique, et un checkbox à côté, avec lequel on peut choisir quels graphiques on veut voir à un moment précis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feedback de chef de projet par rapport à l'avancement du projet, et indeces pour le stockage des données </t>
+  </si>
+  <si>
+    <t>Il faudra prévoir une stratégie pour l'ajout des nouveau données (il faudrait mieux prendre en compte les nouvelles données, si elles se mettent sur le même moment au temps). Également il faudra penser à l'indiquation de ces changement à l'utilisateur (un message pop-up qui prouve la réussite et le nombre de changement au minimum, et idéalement une comparaison des deux graphiques)</t>
+  </si>
+  <si>
+    <t>Vérifier si le graphique avec le même nom existe déjà -&gt; si oui afficher une erreur</t>
+  </si>
+  <si>
+    <t>Réaliser la sauvegarde des données</t>
+  </si>
+  <si>
+    <t>Les données sont sauvegardées dans un fichier .json</t>
+  </si>
+  <si>
+    <t>Documentation jdt</t>
+  </si>
+  <si>
+    <t>Transmision de détails pour le projet par le chef de projet</t>
+  </si>
+  <si>
+    <t>le message transmit: pour obtenir une évaluation à 80% du projet, il faut faire une release cette semaine. Il faudra travailler le système de sauvegarde des données et gestion des données répetitives</t>
+  </si>
+  <si>
+    <t>Correction du dossier de sauvegarde</t>
   </si>
 </sst>
 </file>
@@ -1241,16 +1279,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>195</c:v>
+                  <c:v>230</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>430</c:v>
+                  <c:v>605</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>85</c:v>
+                  <c:v>90</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -2096,16 +2134,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.27464788732394368</c:v>
+                  <c:v>0.24864864864864866</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.60563380281690138</c:v>
+                  <c:v>0.65405405405405403</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.11971830985915492</c:v>
+                  <c:v>9.7297297297297303E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4340,7 +4378,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>11 heures 50 minutes</v>
+        <v>15 heures 25 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4355,15 +4393,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>180</v>
+        <v>300</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>530</v>
+        <v>625</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>710</v>
+        <v>925</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -5033,123 +5071,217 @@
       <c r="G33" s="40"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="62" t="str">
+      <c r="A34" s="62">
         <f>IF(ISBLANK(B34),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B34))</f>
-        <v/>
-      </c>
-      <c r="B34" s="30"/>
+        <v>40</v>
+      </c>
+      <c r="B34" s="30">
+        <v>46294</v>
+      </c>
       <c r="C34" s="31"/>
-      <c r="D34" s="32"/>
-      <c r="E34" s="33"/>
-      <c r="F34" s="22"/>
+      <c r="D34" s="32">
+        <v>5</v>
+      </c>
+      <c r="E34" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" s="22" t="s">
+        <v>64</v>
+      </c>
       <c r="G34" s="39"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="63" t="str">
+    <row r="35" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A35" s="63">
         <f>IF(ISBLANK(B35),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B35))</f>
-        <v/>
-      </c>
-      <c r="B35" s="34"/>
+        <v>40</v>
+      </c>
+      <c r="B35" s="34">
+        <v>46294</v>
+      </c>
       <c r="C35" s="35"/>
-      <c r="D35" s="36"/>
-      <c r="E35" s="37"/>
-      <c r="F35" s="23"/>
-      <c r="G35" s="40"/>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="62" t="str">
+      <c r="D35" s="36">
+        <v>10</v>
+      </c>
+      <c r="E35" s="37" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="G35" s="40" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A36" s="62">
         <f>IF(ISBLANK(B36),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B36))</f>
-        <v/>
-      </c>
-      <c r="B36" s="30"/>
-      <c r="C36" s="31"/>
-      <c r="D36" s="32"/>
-      <c r="E36" s="33"/>
-      <c r="F36" s="22"/>
-      <c r="G36" s="39"/>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="63" t="str">
+        <v>40</v>
+      </c>
+      <c r="B36" s="30">
+        <v>46294</v>
+      </c>
+      <c r="C36" s="31">
+        <v>1</v>
+      </c>
+      <c r="D36" s="32">
+        <v>15</v>
+      </c>
+      <c r="E36" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F36" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="G36" s="39" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="78.75" x14ac:dyDescent="0.25">
+      <c r="A37" s="63">
         <f>IF(ISBLANK(B37),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B37))</f>
-        <v/>
-      </c>
-      <c r="B37" s="34"/>
+        <v>40</v>
+      </c>
+      <c r="B37" s="34">
+        <v>46294</v>
+      </c>
       <c r="C37" s="35"/>
-      <c r="D37" s="36"/>
-      <c r="E37" s="37"/>
-      <c r="F37" s="22"/>
-      <c r="G37" s="40"/>
+      <c r="D37" s="36">
+        <v>15</v>
+      </c>
+      <c r="E37" s="37" t="s">
+        <v>14</v>
+      </c>
+      <c r="F37" s="22" t="s">
+        <v>68</v>
+      </c>
+      <c r="G37" s="40" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" s="62" t="str">
+      <c r="A38" s="62">
         <f>IF(ISBLANK(B38),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B38))</f>
-        <v/>
-      </c>
-      <c r="B38" s="30"/>
+        <v>40</v>
+      </c>
+      <c r="B38" s="30">
+        <v>46294</v>
+      </c>
       <c r="C38" s="31"/>
-      <c r="D38" s="32"/>
-      <c r="E38" s="33"/>
-      <c r="F38" s="22"/>
+      <c r="D38" s="32">
+        <v>10</v>
+      </c>
+      <c r="E38" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F38" s="22" t="s">
+        <v>70</v>
+      </c>
       <c r="G38" s="39"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" s="63" t="str">
+      <c r="A39" s="63">
         <f>IF(ISBLANK(B39),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B39))</f>
-        <v/>
-      </c>
-      <c r="B39" s="34"/>
-      <c r="C39" s="35"/>
-      <c r="D39" s="36"/>
-      <c r="E39" s="37"/>
-      <c r="F39" s="22"/>
-      <c r="G39" s="40"/>
+        <v>40</v>
+      </c>
+      <c r="B39" s="34">
+        <v>46294</v>
+      </c>
+      <c r="C39" s="35">
+        <v>1</v>
+      </c>
+      <c r="D39" s="36">
+        <v>5</v>
+      </c>
+      <c r="E39" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F39" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="G39" s="40" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" s="62" t="str">
+      <c r="A40" s="62">
         <f>IF(ISBLANK(B40),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B40))</f>
-        <v/>
-      </c>
-      <c r="B40" s="30"/>
+        <v>40</v>
+      </c>
+      <c r="B40" s="30">
+        <v>46294</v>
+      </c>
       <c r="C40" s="31"/>
-      <c r="D40" s="32"/>
-      <c r="E40" s="33"/>
-      <c r="F40" s="22"/>
+      <c r="D40" s="32">
+        <v>5</v>
+      </c>
+      <c r="E40" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="F40" s="22" t="s">
+        <v>73</v>
+      </c>
       <c r="G40" s="39"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" s="63" t="str">
+    <row r="41" spans="1:7" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A41" s="63">
         <f>IF(ISBLANK(B41),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B41))</f>
-        <v/>
-      </c>
-      <c r="B41" s="34"/>
+        <v>41</v>
+      </c>
+      <c r="B41" s="34">
+        <v>46300</v>
+      </c>
       <c r="C41" s="35"/>
-      <c r="D41" s="36"/>
-      <c r="E41" s="37"/>
-      <c r="F41" s="22"/>
-      <c r="G41" s="40"/>
+      <c r="D41" s="36">
+        <v>5</v>
+      </c>
+      <c r="E41" s="37" t="s">
+        <v>14</v>
+      </c>
+      <c r="F41" s="22" t="s">
+        <v>74</v>
+      </c>
+      <c r="G41" s="40" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A42" s="62" t="str">
+      <c r="A42" s="62">
         <f>IF(ISBLANK(B42),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B42))</f>
-        <v/>
-      </c>
-      <c r="B42" s="30"/>
+        <v>41</v>
+      </c>
+      <c r="B42" s="30">
+        <v>46300</v>
+      </c>
       <c r="C42" s="31"/>
-      <c r="D42" s="32"/>
-      <c r="E42" s="33"/>
-      <c r="F42" s="22"/>
+      <c r="D42" s="32">
+        <v>10</v>
+      </c>
+      <c r="E42" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F42" s="22" t="s">
+        <v>41</v>
+      </c>
       <c r="G42" s="39"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" s="63" t="str">
+      <c r="A43" s="63">
         <f>IF(ISBLANK(B43),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B43))</f>
-        <v/>
-      </c>
-      <c r="B43" s="34"/>
+        <v>41</v>
+      </c>
+      <c r="B43" s="34">
+        <v>46300</v>
+      </c>
       <c r="C43" s="35"/>
-      <c r="D43" s="36"/>
-      <c r="E43" s="37"/>
-      <c r="F43" s="22"/>
+      <c r="D43" s="36">
+        <v>15</v>
+      </c>
+      <c r="E43" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F43" s="22" t="s">
+        <v>76</v>
+      </c>
       <c r="G43" s="40"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
@@ -11158,11 +11290,11 @@
       </c>
       <c r="B6">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E6,'Journal de travail'!$D$7:$D$532)</f>
-        <v>135</v>
+        <v>170</v>
       </c>
       <c r="C6">
         <f t="shared" ref="C6:C10" si="0">SUM(A6:B6)</f>
-        <v>195</v>
+        <v>230</v>
       </c>
       <c r="E6" s="70" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11170,11 +11302,11 @@
       </c>
       <c r="F6" s="71" t="str">
         <f>QUOTIENT(SUM(A6:B6),60)&amp;" h "&amp;TEXT(MOD(SUM(A6:B6),60), "00")&amp;" min"</f>
-        <v>3 h 15 min</v>
+        <v>3 h 50 min</v>
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.27464788732394368</v>
+        <v>0.24864864864864866</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11191,15 +11323,15 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>310</v>
+        <v>365</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>430</v>
+        <v>605</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11207,11 +11339,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>7 h 10 min</v>
+        <v>10 h 05 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.60563380281690138</v>
+        <v>0.65405405405405403</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11269,11 +11401,11 @@
       </c>
       <c r="B9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$D$7:$D$532)</f>
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="E9" s="77" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11281,11 +11413,11 @@
       </c>
       <c r="F9" s="74" t="str">
         <f t="shared" si="1"/>
-        <v>1 h 25 min</v>
+        <v>1 h 30 min</v>
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.11971830985915492</v>
+        <v>9.7297297297297303E-2</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11337,26 +11469,26 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>180</v>
+        <v>300</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>530</v>
+        <v>625</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>710</v>
+        <v>925</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>11 h 50 min</v>
+        <v>15 h 25 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.13148148148148148</v>
+        <v>0.17129629629629631</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>

</xml_diff>

<commit_message>
feat : réaliser la supression d'une série
</commit_message>
<xml_diff>
--- a/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
+++ b/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\px20umf\Documents\github\PlotThoseLines\docs\jdt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20A08822-01BB-4CF1-A377-F52ADE7891B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C817C52D-9788-4A47-B13E-A135D0CB8F4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="31590" yWindow="1740" windowWidth="21600" windowHeight="11745" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="80">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -272,6 +272,15 @@
   </si>
   <si>
     <t>Correction du dossier de sauvegarde</t>
+  </si>
+  <si>
+    <t>Je commence par l'ajout d'un fichier pour le même graphique, en enchaînant avec la logique de remplacement des anciens points si la nouvelle série contient  des points communs avec l'ancienne.</t>
+  </si>
+  <si>
+    <t>Attribution du nom de graphique par l'accronyme de l'entreprise, implémentation de logique d'ajout d'une autre serie</t>
+  </si>
+  <si>
+    <t>Partie complètement fonctionnelle, si l'ancien et le nouveau graphique ont des données en commun -&gt; celles de dernier sont prises en compte.</t>
   </si>
 </sst>
 </file>
@@ -1282,7 +1291,7 @@
                   <c:v>230</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>605</c:v>
+                  <c:v>675</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2134,16 +2143,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.24864864864864866</c:v>
+                  <c:v>0.23115577889447236</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.65405405405405403</c:v>
+                  <c:v>0.67839195979899503</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>9.7297297297297303E-2</c:v>
+                  <c:v>9.0452261306532666E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4378,7 +4387,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>15 heures 25 minutes</v>
+        <v>16 heures 35 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4393,15 +4402,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>300</v>
+        <v>360</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>625</v>
+        <v>635</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>925</v>
+        <v>995</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -5244,7 +5253,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A42" s="62">
         <f>IF(ISBLANK(B42),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B42))</f>
         <v>41</v>
@@ -5262,7 +5271,9 @@
       <c r="F42" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="G42" s="39"/>
+      <c r="G42" s="39" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="63">
@@ -5284,17 +5295,29 @@
       </c>
       <c r="G43" s="40"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" s="62" t="str">
+    <row r="44" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A44" s="62">
         <f>IF(ISBLANK(B44),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B44))</f>
-        <v/>
-      </c>
-      <c r="B44" s="30"/>
-      <c r="C44" s="31"/>
-      <c r="D44" s="32"/>
-      <c r="E44" s="33"/>
-      <c r="F44" s="22"/>
-      <c r="G44" s="39"/>
+        <v>41</v>
+      </c>
+      <c r="B44" s="30">
+        <v>46300</v>
+      </c>
+      <c r="C44" s="31">
+        <v>1</v>
+      </c>
+      <c r="D44" s="32">
+        <v>10</v>
+      </c>
+      <c r="E44" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F44" s="23" t="s">
+        <v>78</v>
+      </c>
+      <c r="G44" s="39" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="63" t="str">
@@ -11153,7 +11176,7 @@
       <c r="G532" s="39"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="sC8RJl0M6+wONYXsnCTKmcqXUp1ITAlugv/3BW303r/E9HRpDNWm1EDZcYLBlB50SDN+6uVKCZ+hqkZ4Wju+ZA==" saltValue="fNiMxA6H49sg0PxMFstsLQ==" spinCount="100000" sheet="1" insertHyperlinks="0" selectLockedCells="1" sort="0" autoFilter="0"/>
+  <sheetProtection insertHyperlinks="0" selectLockedCells="1" sort="0" autoFilter="0"/>
   <mergeCells count="4">
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="C5:D5"/>
@@ -11306,7 +11329,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.24864864864864866</v>
+        <v>0.23115577889447236</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11323,15 +11346,15 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>365</v>
+        <v>375</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>605</v>
+        <v>675</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11339,11 +11362,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>10 h 05 min</v>
+        <v>11 h 15 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.65405405405405403</v>
+        <v>0.67839195979899503</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11417,7 +11440,7 @@
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>9.7297297297297303E-2</v>
+        <v>9.0452261306532666E-2</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11469,26 +11492,26 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>300</v>
+        <v>360</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>625</v>
+        <v>635</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>925</v>
+        <v>995</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>15 h 25 min</v>
+        <v>16 h 35 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.17129629629629631</v>
+        <v>0.18425925925925926</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>

</xml_diff>

<commit_message>
docs : fix des dates sur le jdt (je me suis trompé en mettant 29.09 au lieu de 28.09)
</commit_message>
<xml_diff>
--- a/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
+++ b/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\px20umf\Documents\github\PlotThoseLines\docs\jdt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C817C52D-9788-4A47-B13E-A135D0CB8F4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{399DCDD1-2760-42C0-971C-6654ED47BEED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31590" yWindow="1740" windowWidth="21600" windowHeight="11745" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="84">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -281,6 +281,18 @@
   </si>
   <si>
     <t>Partie complètement fonctionnelle, si l'ancien et le nouveau graphique ont des données en commun -&gt; celles de dernier sont prises en compte.</t>
+  </si>
+  <si>
+    <t>Suppresion de série de l'affichage et de la mémoire</t>
+  </si>
+  <si>
+    <t>Boutons pout changer le zoom et exporter le graphique en png</t>
+  </si>
+  <si>
+    <t>Formatage des grands nombres</t>
+  </si>
+  <si>
+    <t>Nombres positifs et négatifs</t>
   </si>
 </sst>
 </file>
@@ -1291,7 +1303,7 @@
                   <c:v>230</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>675</c:v>
+                  <c:v>750</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2143,16 +2155,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.23115577889447236</c:v>
+                  <c:v>0.21495327102803738</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.67839195979899503</c:v>
+                  <c:v>0.7009345794392523</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>9.0452261306532666E-2</c:v>
+                  <c:v>8.4112149532710276E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4387,7 +4399,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>16 heures 35 minutes</v>
+        <v>17 heures 50 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4406,11 +4418,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>635</v>
+        <v>710</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>995</v>
+        <v>1070</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -5085,7 +5097,7 @@
         <v>40</v>
       </c>
       <c r="B34" s="30">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="C34" s="31"/>
       <c r="D34" s="32">
@@ -5104,8 +5116,8 @@
         <f>IF(ISBLANK(B35),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B35))</f>
         <v>40</v>
       </c>
-      <c r="B35" s="34">
-        <v>46294</v>
+      <c r="B35" s="30">
+        <v>46293</v>
       </c>
       <c r="C35" s="35"/>
       <c r="D35" s="36">
@@ -5127,7 +5139,7 @@
         <v>40</v>
       </c>
       <c r="B36" s="30">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="C36" s="31">
         <v>1</v>
@@ -5151,7 +5163,7 @@
         <v>40</v>
       </c>
       <c r="B37" s="34">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="C37" s="35"/>
       <c r="D37" s="36">
@@ -5173,7 +5185,7 @@
         <v>40</v>
       </c>
       <c r="B38" s="30">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="C38" s="31"/>
       <c r="D38" s="32">
@@ -5193,7 +5205,7 @@
         <v>40</v>
       </c>
       <c r="B39" s="34">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="C39" s="35">
         <v>1</v>
@@ -5217,7 +5229,7 @@
         <v>40</v>
       </c>
       <c r="B40" s="30">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="C40" s="31"/>
       <c r="D40" s="32">
@@ -5320,40 +5332,66 @@
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A45" s="63" t="str">
+      <c r="A45" s="63">
         <f>IF(ISBLANK(B45),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B45))</f>
-        <v/>
-      </c>
-      <c r="B45" s="34"/>
+        <v>41</v>
+      </c>
+      <c r="B45" s="34">
+        <v>46300</v>
+      </c>
       <c r="C45" s="35"/>
-      <c r="D45" s="36"/>
-      <c r="E45" s="37"/>
-      <c r="F45" s="22"/>
+      <c r="D45" s="36">
+        <v>30</v>
+      </c>
+      <c r="E45" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F45" s="22" t="s">
+        <v>80</v>
+      </c>
       <c r="G45" s="40"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A46" s="62" t="str">
+      <c r="A46" s="62">
         <f>IF(ISBLANK(B46),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B46))</f>
-        <v/>
-      </c>
-      <c r="B46" s="30"/>
+        <v>41</v>
+      </c>
+      <c r="B46" s="30">
+        <v>46300</v>
+      </c>
       <c r="C46" s="31"/>
-      <c r="D46" s="32"/>
-      <c r="E46" s="33"/>
-      <c r="F46" s="22"/>
+      <c r="D46" s="32">
+        <v>25</v>
+      </c>
+      <c r="E46" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F46" s="22" t="s">
+        <v>81</v>
+      </c>
       <c r="G46" s="39"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" s="63" t="str">
+      <c r="A47" s="63">
         <f>IF(ISBLANK(B47),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B47))</f>
-        <v/>
-      </c>
-      <c r="B47" s="34"/>
+        <v>41</v>
+      </c>
+      <c r="B47" s="34">
+        <v>46300</v>
+      </c>
       <c r="C47" s="35"/>
-      <c r="D47" s="36"/>
-      <c r="E47" s="37"/>
-      <c r="F47" s="22"/>
-      <c r="G47" s="40"/>
+      <c r="D47" s="36">
+        <v>20</v>
+      </c>
+      <c r="E47" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F47" s="22" t="s">
+        <v>82</v>
+      </c>
+      <c r="G47" s="40" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="62" t="str">
@@ -11329,7 +11367,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.23115577889447236</v>
+        <v>0.21495327102803738</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11350,11 +11388,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>375</v>
+        <v>450</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>675</v>
+        <v>750</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11362,11 +11400,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>11 h 15 min</v>
+        <v>12 h 30 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.67839195979899503</v>
+        <v>0.7009345794392523</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11440,7 +11478,7 @@
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>9.0452261306532666E-2</v>
+        <v>8.4112149532710276E-2</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11496,22 +11534,22 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>635</v>
+        <v>710</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>995</v>
+        <v>1070</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>16 h 35 min</v>
+        <v>17 h 50 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.18425925925925926</v>
+        <v>0.19814814814814816</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>

</xml_diff>

<commit_message>
docs : màj du jdt
</commit_message>
<xml_diff>
--- a/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
+++ b/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\px20umf\Documents\github\PlotThoseLines\docs\jdt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{399DCDD1-2760-42C0-971C-6654ED47BEED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C012618B-47CD-46C8-82C3-4648B7303650}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -40,8 +40,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="85">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -293,6 +315,9 @@
   </si>
   <si>
     <t>Nombres positifs et négatifs</t>
+  </si>
+  <si>
+    <t>Mise à jour du jdt</t>
   </si>
 </sst>
 </file>
@@ -1309,7 +1334,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>90</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -2155,16 +2180,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.21495327102803738</c:v>
+                  <c:v>0.21296296296296297</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.7009345794392523</c:v>
+                  <c:v>0.69444444444444442</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>8.4112149532710276E-2</c:v>
+                  <c:v>9.2592592592592587E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4399,7 +4424,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>17 heures 50 minutes</v>
+        <v>18 heures 0 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4418,11 +4443,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>710</v>
+        <v>720</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>1070</v>
+        <v>1080</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4586,6 +4611,13 @@
         <v>34</v>
       </c>
       <c r="G11" s="40"/>
+      <c r="I11" t="str" cm="1">
+        <f t="array" ref="I11">_xlfn.LET(
+  _xlpm.tot, SUM((B$7:B$100=B7) * (IFERROR(SUBSTITUTE(C$7:C$100," h","")*60, 0) + IFERROR(SUBSTITUTE(D$7:D$100," min","")*1, 0))),
+  INT(_xlpm.tot/60) &amp; " h " &amp; TEXT(MOD(_xlpm.tot, 60), "00") &amp; " min"
+)</f>
+        <v>2 h 55 min</v>
+      </c>
       <c r="M11" t="s">
         <v>17</v>
       </c>
@@ -5394,15 +5426,23 @@
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="62" t="str">
+      <c r="A48" s="62">
         <f>IF(ISBLANK(B48),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B48))</f>
-        <v/>
-      </c>
-      <c r="B48" s="30"/>
+        <v>41</v>
+      </c>
+      <c r="B48" s="30">
+        <v>46300</v>
+      </c>
       <c r="C48" s="31"/>
-      <c r="D48" s="32"/>
-      <c r="E48" s="33"/>
-      <c r="F48" s="22"/>
+      <c r="D48" s="32">
+        <v>10</v>
+      </c>
+      <c r="E48" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="F48" s="22" t="s">
+        <v>84</v>
+      </c>
       <c r="G48" s="39"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
@@ -11367,7 +11407,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.21495327102803738</v>
+        <v>0.21296296296296297</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11404,7 +11444,7 @@
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.7009345794392523</v>
+        <v>0.69444444444444442</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11462,11 +11502,11 @@
       </c>
       <c r="B9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$D$7:$D$532)</f>
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="E9" s="77" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11474,11 +11514,11 @@
       </c>
       <c r="F9" s="74" t="str">
         <f t="shared" si="1"/>
-        <v>1 h 30 min</v>
+        <v>1 h 40 min</v>
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>8.4112149532710276E-2</v>
+        <v>9.2592592592592587E-2</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11534,22 +11574,22 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>710</v>
+        <v>720</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>1070</v>
+        <v>1080</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>17 h 50 min</v>
+        <v>18 h 00 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.19814814814814816</v>
+        <v>0.2</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>

</xml_diff>

<commit_message>
fix : transformation de boucles foreach dans des méthodes LINQ
</commit_message>
<xml_diff>
--- a/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
+++ b/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="98">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -287,6 +287,9 @@
   </si>
   <si>
     <t>Création de logo et son utilisation dans le projet</t>
+  </si>
+  <si>
+    <t>Ajout de légendes pour chaque axe du graphique</t>
   </si>
   <si>
     <t>Total heures TPI</t>
@@ -891,7 +894,7 @@
                   <c:v>245</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>805</c:v>
+                  <c:v>830</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -1167,16 +1170,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0.21304347826086956</c:v>
+                  <c:v>0.20851063829787234</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.7</c:v>
+                  <c:v>0.7063829787234043</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.08695652173913043</c:v>
+                  <c:v>0.0851063829787234</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -1255,7 +1258,7 @@
       <xdr:col>10</xdr:col>
       <xdr:colOff>203200</xdr:colOff>
       <xdr:row>35</xdr:row>
-      <xdr:rowOff>185836</xdr:rowOff>
+      <xdr:rowOff>185790</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1264,7 +1267,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="0"/>
-        <a:ext cx="5499100" cy="5708604"/>
+        <a:ext cx="5499100" cy="5708558"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1285,7 +1288,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>419100</xdr:colOff>
       <xdr:row>35</xdr:row>
-      <xdr:rowOff>173136</xdr:rowOff>
+      <xdr:rowOff>173090</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1294,7 +1297,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="0"/>
-        <a:ext cx="5572125" cy="5702254"/>
+        <a:ext cx="5572125" cy="5702208"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1534,7 +1537,7 @@
       <c r="B3" s="5"/>
       <c r="C3" s="65" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>19 heures 10 minutes</v>
+        <v>19 heures 35 minutes</v>
       </c>
       <c r="D3" s="16"/>
       <c r="E3" s="3"/>
@@ -1553,11 +1556,11 @@
       </c>
       <c r="D4" s="16">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>790</v>
+        <v>815</v>
       </c>
       <c r="E4" s="16">
         <f>SUM(C4:D4)</f>
-        <v>1150</v>
+        <v>1175</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -2816,19 +2819,27 @@
       </c>
     </row>
     <row r="52" ht="17.18">
-      <c r="A52" s="60" t="str">
+      <c r="A52" s="60">
         <f>IF(ISBLANK(B52),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B52))</f>
-        <v/>
-      </c>
-      <c r="B52" s="28"/>
+        <v>4</v>
+      </c>
+      <c r="B52" s="28">
+        <v>25.1</v>
+      </c>
       <c r="C52" s="29"/>
-      <c r="D52" s="30"/>
-      <c r="E52" s="31"/>
-      <c r="F52" s="21"/>
+      <c r="D52" s="30">
+        <v>25</v>
+      </c>
+      <c r="E52" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="F52" s="21" t="s">
+        <v>86</v>
+      </c>
       <c r="G52" s="37"/>
       <c r="H52" t="str">
         <f>IF(OR(ISBLANK(B52),B52=""),"",IF(B52=B51,"",INT(((SUMIF(B:B,B52,C:C)*60)+SUMIF(B:B,B52,D:D))/60)&amp;" h "&amp;TEXT(MOD((SUMIF(B:B,B52,C:C)*60)+SUMIF(B:B,B52,D:D),60),"00")&amp;" min"))</f>
-        <v/>
+        <v>0 h 25 min</v>
       </c>
     </row>
     <row r="53" ht="17.18">
@@ -10602,13 +10613,13 @@
   <sheetData>
     <row r="2" ht="27.27">
       <c r="E2" s="64" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F2" s="66">
         <v>90</v>
       </c>
       <c r="G2" s="64" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="L2" s="17"/>
       <c r="M2" s="42"/>
@@ -10621,42 +10632,42 @@
     </row>
     <row r="4" ht="27.27">
       <c r="E4" s="64" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="L4" s="64" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="M4" s="39"/>
       <c r="N4" s="18"/>
     </row>
     <row r="5" ht="23.86">
       <c r="A5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C5" s="39" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D5" s="40"/>
       <c r="E5" s="43" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F5" s="44" t="s">
+        <v>95</v>
+      </c>
+      <c r="G5" s="45" t="s">
+        <v>96</v>
+      </c>
+      <c r="L5" s="46" t="s">
         <v>94</v>
       </c>
-      <c r="G5" s="45" t="s">
+      <c r="M5" s="47" t="s">
         <v>95</v>
       </c>
-      <c r="L5" s="46" t="s">
-        <v>93</v>
-      </c>
-      <c r="M5" s="47" t="s">
-        <v>94</v>
-      </c>
       <c r="N5" s="48" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" ht="23.86">
@@ -10682,7 +10693,7 @@
       </c>
       <c r="G6" s="70">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.21304347826086956</v>
+        <v>0.20851063829787234</v>
       </c>
       <c r="L6" s="49" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10703,11 +10714,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>505</v>
+        <v>530</v>
       </c>
       <c r="C7">
         <f>SUM(A7:B7)</f>
-        <v>805</v>
+        <v>830</v>
       </c>
       <c r="E7" s="71" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10715,11 +10726,11 @@
       </c>
       <c r="F7" s="72" t="str">
         <f>QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60),"00")&amp;" min"</f>
-        <v>13 h 25 min</v>
+        <v>13 h 50 min</v>
       </c>
       <c r="G7" s="73">
         <f>SUM(A7:B7)/$C$11</f>
-        <v>0.7</v>
+        <v>0.7063829787234043</v>
       </c>
       <c r="L7" s="51" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10793,7 +10804,7 @@
       </c>
       <c r="G9" s="73">
         <f>SUM(A9:B9)/$C$11</f>
-        <v>0.08695652173913043</v>
+        <v>0.0851063829787234</v>
       </c>
       <c r="L9" s="53" t="str">
         <f>'Journal de travail'!M11</f>
@@ -10849,25 +10860,25 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>790</v>
+        <v>815</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>1150</v>
+        <v>1175</v>
       </c>
       <c r="E11" s="79" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F11" s="69" t="str">
         <f>QUOTIENT(SUM(A11:B11),60)&amp;" h "&amp;TEXT(MOD(SUM(A11:B11),60),"00")&amp;" min"</f>
-        <v>19 h 10 min</v>
+        <v>19 h 35 min</v>
       </c>
       <c r="G11" s="80">
         <f>C11/C12</f>
-        <v>0.21296296296296297</v>
+        <v>0.2175925925925926</v>
       </c>
       <c r="L11" s="54" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="M11" s="55"/>
       <c r="N11" s="58">

</xml_diff>

<commit_message>
feat : déplacement de la logique de parser des csv dans une classe séparée
</commit_message>
<xml_diff>
--- a/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
+++ b/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="102">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -290,6 +290,18 @@
   </si>
   <si>
     <t>Ajout de légendes pour chaque axe du graphique</t>
+  </si>
+  <si>
+    <t>Analyse du feedback du chef de projet</t>
+  </si>
+  <si>
+    <t>Je me suis un peu trop concentré sur l'intéraction et le visuel du programme, en oubliant certains point critiques, comme l'ajout des tests, utilisation de LINQ et une bonne organisation des méthodes (il faut créer des classes séparées pour chaque méthode important)</t>
+  </si>
+  <si>
+    <t>Transformation des boucles foreach en méthodes LINQ</t>
+  </si>
+  <si>
+    <t>Déplacement de la logique de parser des csv dans une classe séparée</t>
   </si>
   <si>
     <t>Total heures TPI</t>
@@ -891,10 +903,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>245</c:v>
+                  <c:v>265</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>830</c:v>
+                  <c:v>910</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -1170,16 +1182,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0.20851063829787234</c:v>
+                  <c:v>0.20784313725490197</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.7063829787234043</c:v>
+                  <c:v>0.7137254901960784</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.0851063829787234</c:v>
+                  <c:v>0.0784313725490196</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -1258,7 +1270,7 @@
       <xdr:col>10</xdr:col>
       <xdr:colOff>203200</xdr:colOff>
       <xdr:row>35</xdr:row>
-      <xdr:rowOff>185790</xdr:rowOff>
+      <xdr:rowOff>185744</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1267,7 +1279,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="0"/>
-        <a:ext cx="5499100" cy="5708558"/>
+        <a:ext cx="5499100" cy="5708512"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1288,7 +1300,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>419100</xdr:colOff>
       <xdr:row>35</xdr:row>
-      <xdr:rowOff>173090</xdr:rowOff>
+      <xdr:rowOff>173044</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1297,7 +1309,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="0"/>
-        <a:ext cx="5572125" cy="5702208"/>
+        <a:ext cx="5572125" cy="5702162"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1537,7 +1549,7 @@
       <c r="B3" s="5"/>
       <c r="C3" s="65" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>19 heures 35 minutes</v>
+        <v>21 heures 15 minutes</v>
       </c>
       <c r="D3" s="16"/>
       <c r="E3" s="3"/>
@@ -1556,11 +1568,11 @@
       </c>
       <c r="D4" s="16">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>815</v>
+        <v>915</v>
       </c>
       <c r="E4" s="16">
         <f>SUM(C4:D4)</f>
-        <v>1175</v>
+        <v>1275</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -2821,10 +2833,10 @@
     <row r="52" ht="17.18">
       <c r="A52" s="60">
         <f>IF(ISBLANK(B52),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B52))</f>
-        <v>4</v>
+        <v>43</v>
       </c>
       <c r="B52" s="28">
-        <v>25.1</v>
+        <v>46320</v>
       </c>
       <c r="C52" s="29"/>
       <c r="D52" s="30">
@@ -2839,35 +2851,53 @@
       <c r="G52" s="37"/>
       <c r="H52" t="str">
         <f>IF(OR(ISBLANK(B52),B52=""),"",IF(B52=B51,"",INT(((SUMIF(B:B,B52,C:C)*60)+SUMIF(B:B,B52,D:D))/60)&amp;" h "&amp;TEXT(MOD((SUMIF(B:B,B52,C:C)*60)+SUMIF(B:B,B52,D:D),60),"00")&amp;" min"))</f>
-        <v>0 h 25 min</v>
-      </c>
-    </row>
-    <row r="53" ht="17.18">
-      <c r="A53" s="61" t="str">
+        <v>2 h 05 min</v>
+      </c>
+    </row>
+    <row r="53" ht="77.25">
+      <c r="A53" s="61">
         <f>IF(ISBLANK(B53),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B53))</f>
-        <v/>
-      </c>
-      <c r="B53" s="32"/>
+        <v>43</v>
+      </c>
+      <c r="B53" s="28">
+        <v>46320</v>
+      </c>
       <c r="C53" s="33"/>
-      <c r="D53" s="34"/>
-      <c r="E53" s="35"/>
-      <c r="F53" s="21"/>
-      <c r="G53" s="38"/>
+      <c r="D53" s="34">
+        <v>20</v>
+      </c>
+      <c r="E53" s="35" t="s">
+        <v>18</v>
+      </c>
+      <c r="F53" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="G53" s="38" t="s">
+        <v>88</v>
+      </c>
       <c r="H53" t="str">
         <f>IF(OR(ISBLANK(B53),B53=""),"",IF(B53=B52,"",INT(((SUMIF(B:B,B53,C:C)*60)+SUMIF(B:B,B53,D:D))/60)&amp;" h "&amp;TEXT(MOD((SUMIF(B:B,B53,C:C)*60)+SUMIF(B:B,B53,D:D),60),"00")&amp;" min"))</f>
         <v/>
       </c>
     </row>
     <row r="54" ht="17.18">
-      <c r="A54" s="60" t="str">
+      <c r="A54" s="60">
         <f>IF(ISBLANK(B54),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B54))</f>
-        <v/>
-      </c>
-      <c r="B54" s="28"/>
+        <v>43</v>
+      </c>
+      <c r="B54" s="28">
+        <v>46320</v>
+      </c>
       <c r="C54" s="29"/>
-      <c r="D54" s="30"/>
-      <c r="E54" s="31"/>
-      <c r="F54" s="21"/>
+      <c r="D54" s="30">
+        <v>50</v>
+      </c>
+      <c r="E54" s="35" t="s">
+        <v>22</v>
+      </c>
+      <c r="F54" s="21" t="s">
+        <v>89</v>
+      </c>
       <c r="G54" s="37"/>
       <c r="H54" t="str">
         <f>IF(OR(ISBLANK(B54),B54=""),"",IF(B54=B53,"",INT(((SUMIF(B:B,B54,C:C)*60)+SUMIF(B:B,B54,D:D))/60)&amp;" h "&amp;TEXT(MOD((SUMIF(B:B,B54,C:C)*60)+SUMIF(B:B,B54,D:D),60),"00")&amp;" min"))</f>
@@ -2875,15 +2905,23 @@
       </c>
     </row>
     <row r="55" ht="17.18">
-      <c r="A55" s="61" t="str">
+      <c r="A55" s="61">
         <f>IF(ISBLANK(B55),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B55))</f>
-        <v/>
-      </c>
-      <c r="B55" s="32"/>
+        <v>43</v>
+      </c>
+      <c r="B55" s="28">
+        <v>46320</v>
+      </c>
       <c r="C55" s="33"/>
-      <c r="D55" s="34"/>
-      <c r="E55" s="35"/>
-      <c r="F55" s="21"/>
+      <c r="D55" s="34">
+        <v>30</v>
+      </c>
+      <c r="E55" s="35" t="s">
+        <v>22</v>
+      </c>
+      <c r="F55" s="21" t="s">
+        <v>90</v>
+      </c>
       <c r="G55" s="38"/>
       <c r="H55" t="str">
         <f>IF(OR(ISBLANK(B55),B55=""),"",IF(B55=B54,"",INT(((SUMIF(B:B,B55,C:C)*60)+SUMIF(B:B,B55,D:D))/60)&amp;" h "&amp;TEXT(MOD((SUMIF(B:B,B55,C:C)*60)+SUMIF(B:B,B55,D:D),60),"00")&amp;" min"))</f>
@@ -10574,15 +10612,24 @@
       <formula>$E7="Implémentation"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C7:C532">
+  <dataValidations count="6">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C7:C53 C55:C532">
       <formula1>$N$7:$N$15</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D7:D532">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D7:D53 D55:D532">
       <formula1>$O$7:$O$19</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E7:E532">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E7:E53 E55:E532">
       <formula1>$M$7:$M$12</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E54">
+      <formula1>$M$7:$M$12</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C54">
+      <formula1>$N$7:$N$15</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D54">
+      <formula1>$O$7:$O$19</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.699999988079071" right="0.699999988079071" top="0.75" bottom="0.75" header="0.30000001192092896" footer="0.30000001192092896"/>
@@ -10613,13 +10660,13 @@
   <sheetData>
     <row r="2" ht="27.27">
       <c r="E2" s="64" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="F2" s="66">
         <v>90</v>
       </c>
       <c r="G2" s="64" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="L2" s="17"/>
       <c r="M2" s="42"/>
@@ -10632,42 +10679,42 @@
     </row>
     <row r="4" ht="27.27">
       <c r="E4" s="64" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="L4" s="64" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="M4" s="39"/>
       <c r="N4" s="18"/>
     </row>
     <row r="5" ht="23.86">
       <c r="A5" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B5" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C5" s="39" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D5" s="40"/>
       <c r="E5" s="43" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="F5" s="44" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="G5" s="45" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="L5" s="46" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="M5" s="47" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="N5" s="48" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" ht="23.86">
@@ -10677,11 +10724,11 @@
       </c>
       <c r="B6">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E6,'Journal de travail'!$D$7:$D$532)</f>
-        <v>185</v>
+        <v>205</v>
       </c>
       <c r="C6">
         <f>SUM(A6:B6)</f>
-        <v>245</v>
+        <v>265</v>
       </c>
       <c r="E6" s="68" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10689,11 +10736,11 @@
       </c>
       <c r="F6" s="69" t="str">
         <f>QUOTIENT(SUM(A6:B6),60)&amp;" h "&amp;TEXT(MOD(SUM(A6:B6),60),"00")&amp;" min"</f>
-        <v>4 h 05 min</v>
+        <v>4 h 25 min</v>
       </c>
       <c r="G6" s="70">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.20851063829787234</v>
+        <v>0.20784313725490197</v>
       </c>
       <c r="L6" s="49" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10714,11 +10761,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>530</v>
+        <v>610</v>
       </c>
       <c r="C7">
         <f>SUM(A7:B7)</f>
-        <v>830</v>
+        <v>910</v>
       </c>
       <c r="E7" s="71" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10726,11 +10773,11 @@
       </c>
       <c r="F7" s="72" t="str">
         <f>QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60),"00")&amp;" min"</f>
-        <v>13 h 50 min</v>
+        <v>15 h 10 min</v>
       </c>
       <c r="G7" s="73">
         <f>SUM(A7:B7)/$C$11</f>
-        <v>0.7063829787234043</v>
+        <v>0.7137254901960784</v>
       </c>
       <c r="L7" s="51" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10804,7 +10851,7 @@
       </c>
       <c r="G9" s="73">
         <f>SUM(A9:B9)/$C$11</f>
-        <v>0.0851063829787234</v>
+        <v>0.0784313725490196</v>
       </c>
       <c r="L9" s="53" t="str">
         <f>'Journal de travail'!M11</f>
@@ -10860,25 +10907,25 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>815</v>
+        <v>915</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>1175</v>
+        <v>1275</v>
       </c>
       <c r="E11" s="79" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="F11" s="69" t="str">
         <f>QUOTIENT(SUM(A11:B11),60)&amp;" h "&amp;TEXT(MOD(SUM(A11:B11),60),"00")&amp;" min"</f>
-        <v>19 h 35 min</v>
+        <v>21 h 15 min</v>
       </c>
       <c r="G11" s="80">
         <f>C11/C12</f>
-        <v>0.2175925925925926</v>
+        <v>0.2361111111111111</v>
       </c>
       <c r="L11" s="54" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="M11" s="55"/>
       <c r="N11" s="58">

</xml_diff>

<commit_message>
feat : déplacement de la logique de transformation des nombres dans une classe séparée
</commit_message>
<xml_diff>
--- a/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
+++ b/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="103">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -302,6 +302,9 @@
   </si>
   <si>
     <t>Déplacement de la logique de parser des csv dans une classe séparée</t>
+  </si>
+  <si>
+    <t>Déplacement de la logique de transformation des nombres dans une classe séparée</t>
   </si>
   <si>
     <t>Total heures TPI</t>
@@ -906,7 +909,7 @@
                   <c:v>265</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>910</c:v>
+                  <c:v>915</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -1182,16 +1185,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0.20784313725490197</c:v>
+                  <c:v>0.20703125</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.7137254901960784</c:v>
+                  <c:v>0.71484375</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.0784313725490196</c:v>
+                  <c:v>0.078125</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -1549,7 +1552,7 @@
       <c r="B3" s="5"/>
       <c r="C3" s="65" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>21 heures 15 minutes</v>
+        <v>21 heures 20 minutes</v>
       </c>
       <c r="D3" s="16"/>
       <c r="E3" s="3"/>
@@ -1568,11 +1571,11 @@
       </c>
       <c r="D4" s="16">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>915</v>
+        <v>920</v>
       </c>
       <c r="E4" s="16">
         <f>SUM(C4:D4)</f>
-        <v>1275</v>
+        <v>1280</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -2851,7 +2854,7 @@
       <c r="G52" s="37"/>
       <c r="H52" t="str">
         <f>IF(OR(ISBLANK(B52),B52=""),"",IF(B52=B51,"",INT(((SUMIF(B:B,B52,C:C)*60)+SUMIF(B:B,B52,D:D))/60)&amp;" h "&amp;TEXT(MOD((SUMIF(B:B,B52,C:C)*60)+SUMIF(B:B,B52,D:D),60),"00")&amp;" min"))</f>
-        <v>2 h 05 min</v>
+        <v>2 h 10 min</v>
       </c>
     </row>
     <row r="53" ht="77.25">
@@ -2929,15 +2932,23 @@
       </c>
     </row>
     <row r="56" ht="17.18">
-      <c r="A56" s="60" t="str">
+      <c r="A56" s="60">
         <f>IF(ISBLANK(B56),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B56))</f>
-        <v/>
-      </c>
-      <c r="B56" s="28"/>
+        <v>43</v>
+      </c>
+      <c r="B56" s="28">
+        <v>46320</v>
+      </c>
       <c r="C56" s="29"/>
-      <c r="D56" s="30"/>
-      <c r="E56" s="31"/>
-      <c r="F56" s="37"/>
+      <c r="D56" s="30">
+        <v>5</v>
+      </c>
+      <c r="E56" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="F56" s="21" t="s">
+        <v>91</v>
+      </c>
       <c r="G56" s="37"/>
       <c r="H56" t="str">
         <f>IF(OR(ISBLANK(B56),B56=""),"",IF(B56=B55,"",INT(((SUMIF(B:B,B56,C:C)*60)+SUMIF(B:B,B56,D:D))/60)&amp;" h "&amp;TEXT(MOD((SUMIF(B:B,B56,C:C)*60)+SUMIF(B:B,B56,D:D),60),"00")&amp;" min"))</f>
@@ -10660,13 +10671,13 @@
   <sheetData>
     <row r="2" ht="27.27">
       <c r="E2" s="64" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F2" s="66">
         <v>90</v>
       </c>
       <c r="G2" s="64" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="L2" s="17"/>
       <c r="M2" s="42"/>
@@ -10679,42 +10690,42 @@
     </row>
     <row r="4" ht="27.27">
       <c r="E4" s="64" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="L4" s="64" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="M4" s="39"/>
       <c r="N4" s="18"/>
     </row>
     <row r="5" ht="23.86">
       <c r="A5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C5" s="39" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D5" s="40"/>
       <c r="E5" s="43" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F5" s="44" t="s">
+        <v>100</v>
+      </c>
+      <c r="G5" s="45" t="s">
+        <v>101</v>
+      </c>
+      <c r="L5" s="46" t="s">
         <v>99</v>
       </c>
-      <c r="G5" s="45" t="s">
+      <c r="M5" s="47" t="s">
         <v>100</v>
       </c>
-      <c r="L5" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="M5" s="47" t="s">
-        <v>99</v>
-      </c>
       <c r="N5" s="48" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="6" ht="23.86">
@@ -10740,7 +10751,7 @@
       </c>
       <c r="G6" s="70">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.20784313725490197</v>
+        <v>0.20703125</v>
       </c>
       <c r="L6" s="49" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10761,11 +10772,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>610</v>
+        <v>615</v>
       </c>
       <c r="C7">
         <f>SUM(A7:B7)</f>
-        <v>910</v>
+        <v>915</v>
       </c>
       <c r="E7" s="71" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10773,11 +10784,11 @@
       </c>
       <c r="F7" s="72" t="str">
         <f>QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60),"00")&amp;" min"</f>
-        <v>15 h 10 min</v>
+        <v>15 h 15 min</v>
       </c>
       <c r="G7" s="73">
         <f>SUM(A7:B7)/$C$11</f>
-        <v>0.7137254901960784</v>
+        <v>0.71484375</v>
       </c>
       <c r="L7" s="51" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10851,7 +10862,7 @@
       </c>
       <c r="G9" s="73">
         <f>SUM(A9:B9)/$C$11</f>
-        <v>0.0784313725490196</v>
+        <v>0.078125</v>
       </c>
       <c r="L9" s="53" t="str">
         <f>'Journal de travail'!M11</f>
@@ -10907,25 +10918,25 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>915</v>
+        <v>920</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>1275</v>
+        <v>1280</v>
       </c>
       <c r="E11" s="79" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F11" s="69" t="str">
         <f>QUOTIENT(SUM(A11:B11),60)&amp;" h "&amp;TEXT(MOD(SUM(A11:B11),60),"00")&amp;" min"</f>
-        <v>21 h 15 min</v>
+        <v>21 h 20 min</v>
       </c>
       <c r="G11" s="80">
         <f>C11/C12</f>
-        <v>0.2361111111111111</v>
+        <v>0.23703703703703705</v>
       </c>
       <c r="L11" s="54" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M11" s="55"/>
       <c r="N11" s="58">

</xml_diff>

<commit_message>
feat : déplacement de la logique de merge des séries dans une classe séparée
</commit_message>
<xml_diff>
--- a/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
+++ b/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="104">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -305,6 +305,9 @@
   </si>
   <si>
     <t>Déplacement de la logique de transformation des nombres dans une classe séparée</t>
+  </si>
+  <si>
+    <t>Déplacement de la logique de merge des séries dans une classe séparée</t>
   </si>
   <si>
     <t>Total heures TPI</t>
@@ -909,7 +912,7 @@
                   <c:v>265</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>915</c:v>
+                  <c:v>945</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -1185,16 +1188,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0.20703125</c:v>
+                  <c:v>0.20229007633587787</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.71484375</c:v>
+                  <c:v>0.7213740458015268</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.078125</c:v>
+                  <c:v>0.07633587786259542</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -1552,7 +1555,7 @@
       <c r="B3" s="5"/>
       <c r="C3" s="65" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>21 heures 20 minutes</v>
+        <v>21 heures 50 minutes</v>
       </c>
       <c r="D3" s="16"/>
       <c r="E3" s="3"/>
@@ -1571,11 +1574,11 @@
       </c>
       <c r="D4" s="16">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>920</v>
+        <v>950</v>
       </c>
       <c r="E4" s="16">
         <f>SUM(C4:D4)</f>
-        <v>1280</v>
+        <v>1310</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -2854,7 +2857,7 @@
       <c r="G52" s="37"/>
       <c r="H52" t="str">
         <f>IF(OR(ISBLANK(B52),B52=""),"",IF(B52=B51,"",INT(((SUMIF(B:B,B52,C:C)*60)+SUMIF(B:B,B52,D:D))/60)&amp;" h "&amp;TEXT(MOD((SUMIF(B:B,B52,C:C)*60)+SUMIF(B:B,B52,D:D),60),"00")&amp;" min"))</f>
-        <v>2 h 10 min</v>
+        <v>2 h 40 min</v>
       </c>
     </row>
     <row r="53" ht="77.25">
@@ -2956,15 +2959,23 @@
       </c>
     </row>
     <row r="57" ht="17.18">
-      <c r="A57" s="61" t="str">
+      <c r="A57" s="61">
         <f>IF(ISBLANK(B57),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B57))</f>
-        <v/>
-      </c>
-      <c r="B57" s="32"/>
+        <v>43</v>
+      </c>
+      <c r="B57" s="28">
+        <v>46320</v>
+      </c>
       <c r="C57" s="33"/>
-      <c r="D57" s="34"/>
-      <c r="E57" s="35"/>
-      <c r="F57" s="38"/>
+      <c r="D57" s="34">
+        <v>30</v>
+      </c>
+      <c r="E57" s="35" t="s">
+        <v>22</v>
+      </c>
+      <c r="F57" s="21" t="s">
+        <v>92</v>
+      </c>
       <c r="G57" s="38"/>
       <c r="H57" t="str">
         <f>IF(OR(ISBLANK(B57),B57=""),"",IF(B57=B56,"",INT(((SUMIF(B:B,B57,C:C)*60)+SUMIF(B:B,B57,D:D))/60)&amp;" h "&amp;TEXT(MOD((SUMIF(B:B,B57,C:C)*60)+SUMIF(B:B,B57,D:D),60),"00")&amp;" min"))</f>
@@ -10623,14 +10634,14 @@
       <formula>$E7="Implémentation"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C7:C53 C55:C532">
+  <dataValidations count="9">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C7:C53 C55:C56 C58:C532">
       <formula1>$N$7:$N$15</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D7:D53 D55:D532">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D7:D53 D55:D56 D58:D532">
       <formula1>$O$7:$O$19</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E7:E53 E55:E532">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E7:E53 E55:E56 E58:E532">
       <formula1>$M$7:$M$12</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E54">
@@ -10641,6 +10652,15 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D54">
       <formula1>$O$7:$O$19</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C57">
+      <formula1>$N$7:$N$15</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D57">
+      <formula1>$O$7:$O$19</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E57">
+      <formula1>$M$7:$M$12</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.699999988079071" right="0.699999988079071" top="0.75" bottom="0.75" header="0.30000001192092896" footer="0.30000001192092896"/>
@@ -10671,13 +10691,13 @@
   <sheetData>
     <row r="2" ht="27.27">
       <c r="E2" s="64" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F2" s="66">
         <v>90</v>
       </c>
       <c r="G2" s="64" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="L2" s="17"/>
       <c r="M2" s="42"/>
@@ -10690,42 +10710,42 @@
     </row>
     <row r="4" ht="27.27">
       <c r="E4" s="64" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="L4" s="64" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="M4" s="39"/>
       <c r="N4" s="18"/>
     </row>
     <row r="5" ht="23.86">
       <c r="A5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C5" s="39" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D5" s="40"/>
       <c r="E5" s="43" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F5" s="44" t="s">
+        <v>101</v>
+      </c>
+      <c r="G5" s="45" t="s">
+        <v>102</v>
+      </c>
+      <c r="L5" s="46" t="s">
         <v>100</v>
       </c>
-      <c r="G5" s="45" t="s">
+      <c r="M5" s="47" t="s">
         <v>101</v>
       </c>
-      <c r="L5" s="46" t="s">
-        <v>99</v>
-      </c>
-      <c r="M5" s="47" t="s">
-        <v>100</v>
-      </c>
       <c r="N5" s="48" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="6" ht="23.86">
@@ -10751,7 +10771,7 @@
       </c>
       <c r="G6" s="70">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.20703125</v>
+        <v>0.20229007633587787</v>
       </c>
       <c r="L6" s="49" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10772,11 +10792,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>615</v>
+        <v>645</v>
       </c>
       <c r="C7">
         <f>SUM(A7:B7)</f>
-        <v>915</v>
+        <v>945</v>
       </c>
       <c r="E7" s="71" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10784,11 +10804,11 @@
       </c>
       <c r="F7" s="72" t="str">
         <f>QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60),"00")&amp;" min"</f>
-        <v>15 h 15 min</v>
+        <v>15 h 45 min</v>
       </c>
       <c r="G7" s="73">
         <f>SUM(A7:B7)/$C$11</f>
-        <v>0.71484375</v>
+        <v>0.7213740458015268</v>
       </c>
       <c r="L7" s="51" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10862,7 +10882,7 @@
       </c>
       <c r="G9" s="73">
         <f>SUM(A9:B9)/$C$11</f>
-        <v>0.078125</v>
+        <v>0.07633587786259542</v>
       </c>
       <c r="L9" s="53" t="str">
         <f>'Journal de travail'!M11</f>
@@ -10918,25 +10938,25 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>920</v>
+        <v>950</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>1280</v>
+        <v>1310</v>
       </c>
       <c r="E11" s="79" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F11" s="69" t="str">
         <f>QUOTIENT(SUM(A11:B11),60)&amp;" h "&amp;TEXT(MOD(SUM(A11:B11),60),"00")&amp;" min"</f>
-        <v>21 h 20 min</v>
+        <v>21 h 50 min</v>
       </c>
       <c r="G11" s="80">
         <f>C11/C12</f>
-        <v>0.23703703703703705</v>
+        <v>0.24259259259259258</v>
       </c>
       <c r="L11" s="54" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="M11" s="55"/>
       <c r="N11" s="58">

</xml_diff>

<commit_message>
docs : màj rapport
</commit_message>
<xml_diff>
--- a/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
+++ b/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\px20umf\Documents\github\PlotThoseLines\docs\jdt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38C2DBAE-5E4F-49C1-931A-8B4B87546635}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85DB7A06-2284-4737-B7B8-E09F3D9F734E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32235" yWindow="2025" windowWidth="21600" windowHeight="11745" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4725" yWindow="1155" windowWidth="21600" windowHeight="11745" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,6 @@
     <sheet name="Initiale VS Effective" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -36,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="115">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -366,6 +365,21 @@
   </si>
   <si>
     <t>pour 26.10</t>
+  </si>
+  <si>
+    <t>Création des tests pour le Parser et le SeriesMerger</t>
+  </si>
+  <si>
+    <t>Disscution sur l'avancement du projet et sur certaines parties du code avec le chef de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mise à jour du rapport </t>
+  </si>
+  <si>
+    <t>Analyse des points restants, il faut encore finir le rapport</t>
+  </si>
+  <si>
+    <t>J'ai completé les bilans dans le rapport</t>
   </si>
 </sst>
 </file>
@@ -1262,16 +1276,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.19354838709677419</c:v>
+                  <c:v>0.18471337579617833</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.73476702508960579</c:v>
+                  <c:v>0.75159235668789814</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>7.1684587813620068E-2</c:v>
+                  <c:v>6.3694267515923567E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1655,7 +1669,7 @@
       <c r="B3" s="85"/>
       <c r="C3" s="65" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>23 heures 15 minutes</v>
+        <v>26 heures 10 minutes</v>
       </c>
       <c r="D3" s="16"/>
       <c r="E3" s="3"/>
@@ -1670,15 +1684,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="16">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>420</v>
+        <v>480</v>
       </c>
       <c r="D4" s="16">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>975</v>
+        <v>1090</v>
       </c>
       <c r="E4" s="16">
         <f>SUM(C4:D4)</f>
-        <v>1395</v>
+        <v>1570</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -3109,7 +3123,7 @@
       <c r="G58" s="37"/>
       <c r="H58" t="str">
         <f t="shared" si="0"/>
-        <v>1 h 25 min</v>
+        <v>3 h 00 min</v>
       </c>
       <c r="I58" t="s">
         <v>109</v>
@@ -3144,15 +3158,23 @@
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A60" s="60" t="str">
+      <c r="A60" s="60">
         <f>IF(ISBLANK(B60),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B60))</f>
-        <v/>
-      </c>
-      <c r="B60" s="28"/>
+        <v>44</v>
+      </c>
+      <c r="B60" s="28">
+        <v>46321</v>
+      </c>
       <c r="C60" s="29"/>
-      <c r="D60" s="30"/>
-      <c r="E60" s="31"/>
-      <c r="F60" s="37"/>
+      <c r="D60" s="30">
+        <v>30</v>
+      </c>
+      <c r="E60" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="F60" s="37" t="s">
+        <v>110</v>
+      </c>
       <c r="G60" s="37"/>
       <c r="H60" t="str">
         <f t="shared" si="0"/>
@@ -3160,15 +3182,23 @@
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A61" s="61" t="str">
+      <c r="A61" s="61">
         <f>IF(ISBLANK(B61),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B61))</f>
-        <v/>
-      </c>
-      <c r="B61" s="32"/>
+        <v>44</v>
+      </c>
+      <c r="B61" s="32">
+        <v>46321</v>
+      </c>
       <c r="C61" s="33"/>
-      <c r="D61" s="34"/>
-      <c r="E61" s="35"/>
-      <c r="F61" s="38"/>
+      <c r="D61" s="34">
+        <v>10</v>
+      </c>
+      <c r="E61" s="35" t="s">
+        <v>18</v>
+      </c>
+      <c r="F61" s="38" t="s">
+        <v>111</v>
+      </c>
       <c r="G61" s="38"/>
       <c r="H61" t="str">
         <f t="shared" si="0"/>
@@ -3176,15 +3206,23 @@
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A62" s="60" t="str">
+      <c r="A62" s="60">
         <f>IF(ISBLANK(B62),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B62))</f>
-        <v/>
-      </c>
-      <c r="B62" s="28"/>
+        <v>44</v>
+      </c>
+      <c r="B62" s="28">
+        <v>46321</v>
+      </c>
       <c r="C62" s="29"/>
-      <c r="D62" s="30"/>
-      <c r="E62" s="31"/>
-      <c r="F62" s="37"/>
+      <c r="D62" s="30">
+        <v>50</v>
+      </c>
+      <c r="E62" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="F62" s="37" t="s">
+        <v>112</v>
+      </c>
       <c r="G62" s="37"/>
       <c r="H62" t="str">
         <f t="shared" si="0"/>
@@ -3192,15 +3230,23 @@
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A63" s="61" t="str">
+      <c r="A63" s="61">
         <f>IF(ISBLANK(B63),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B63))</f>
-        <v/>
-      </c>
-      <c r="B63" s="32"/>
+        <v>44</v>
+      </c>
+      <c r="B63" s="32">
+        <v>46321</v>
+      </c>
       <c r="C63" s="33"/>
-      <c r="D63" s="34"/>
-      <c r="E63" s="35"/>
-      <c r="F63" s="38"/>
+      <c r="D63" s="34">
+        <v>5</v>
+      </c>
+      <c r="E63" s="35" t="s">
+        <v>22</v>
+      </c>
+      <c r="F63" s="38" t="s">
+        <v>81</v>
+      </c>
       <c r="G63" s="38"/>
       <c r="H63" t="str">
         <f t="shared" si="0"/>
@@ -3208,32 +3254,54 @@
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A64" s="60" t="str">
+      <c r="A64" s="60">
         <f>IF(ISBLANK(B64),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B64))</f>
-        <v/>
-      </c>
-      <c r="B64" s="28"/>
+        <v>44</v>
+      </c>
+      <c r="B64" s="28">
+        <v>46323</v>
+      </c>
       <c r="C64" s="29"/>
-      <c r="D64" s="30"/>
-      <c r="E64" s="31"/>
-      <c r="F64" s="37"/>
-      <c r="G64" s="37"/>
+      <c r="D64" s="30">
+        <v>10</v>
+      </c>
+      <c r="E64" s="31" t="s">
+        <v>18</v>
+      </c>
+      <c r="F64" s="37" t="s">
+        <v>32</v>
+      </c>
+      <c r="G64" s="37" t="s">
+        <v>113</v>
+      </c>
       <c r="H64" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>1 h 20 min</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A65" s="61" t="str">
+      <c r="A65" s="61">
         <f>IF(ISBLANK(B65),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B65))</f>
-        <v/>
-      </c>
-      <c r="B65" s="32"/>
-      <c r="C65" s="33"/>
-      <c r="D65" s="34"/>
-      <c r="E65" s="35"/>
-      <c r="F65" s="38"/>
-      <c r="G65" s="38"/>
+        <v>44</v>
+      </c>
+      <c r="B65" s="32">
+        <v>46323</v>
+      </c>
+      <c r="C65" s="33">
+        <v>1</v>
+      </c>
+      <c r="D65" s="34">
+        <v>10</v>
+      </c>
+      <c r="E65" s="35" t="s">
+        <v>22</v>
+      </c>
+      <c r="F65" s="38" t="s">
+        <v>112</v>
+      </c>
+      <c r="G65" s="38" t="s">
+        <v>114</v>
+      </c>
       <c r="H65" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -10850,11 +10918,11 @@
       </c>
       <c r="B6">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E6,'Journal de travail'!$D$7:$D$532)</f>
-        <v>210</v>
+        <v>230</v>
       </c>
       <c r="C6">
         <f t="shared" ref="C6:C11" si="0">SUM(A6:B6)</f>
-        <v>270</v>
+        <v>290</v>
       </c>
       <c r="E6" s="68" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10862,11 +10930,11 @@
       </c>
       <c r="F6" s="69" t="str">
         <f t="shared" ref="F6:F11" si="1">QUOTIENT(SUM(A6:B6),60)&amp;" h "&amp;TEXT(MOD(SUM(A6:B6),60),"00")&amp;" min"</f>
-        <v>4 h 30 min</v>
+        <v>4 h 50 min</v>
       </c>
       <c r="G6" s="70">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.19354838709677419</v>
+        <v>0.18471337579617833</v>
       </c>
       <c r="L6" s="49" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10883,15 +10951,15 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>360</v>
+        <v>420</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>665</v>
+        <v>760</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>1025</v>
+        <v>1180</v>
       </c>
       <c r="E7" s="71" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10899,11 +10967,11 @@
       </c>
       <c r="F7" s="72" t="str">
         <f t="shared" si="1"/>
-        <v>17 h 05 min</v>
+        <v>19 h 40 min</v>
       </c>
       <c r="G7" s="73">
         <f>SUM(A7:B7)/$C$11</f>
-        <v>0.73476702508960579</v>
+        <v>0.75159235668789814</v>
       </c>
       <c r="L7" s="51" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10977,7 +11045,7 @@
       </c>
       <c r="G9" s="73">
         <f>SUM(A9:B9)/$C$11</f>
-        <v>7.1684587813620068E-2</v>
+        <v>6.3694267515923567E-2</v>
       </c>
       <c r="L9" s="53" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11029,26 +11097,26 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>420</v>
+        <v>480</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>975</v>
+        <v>1090</v>
       </c>
       <c r="C11">
         <f t="shared" si="0"/>
-        <v>1395</v>
+        <v>1570</v>
       </c>
       <c r="E11" s="79" t="s">
         <v>103</v>
       </c>
       <c r="F11" s="69" t="str">
         <f t="shared" si="1"/>
-        <v>23 h 15 min</v>
+        <v>26 h 10 min</v>
       </c>
       <c r="G11" s="80">
         <f>C11/C12</f>
-        <v>0.25833333333333336</v>
+        <v>0.29074074074074074</v>
       </c>
       <c r="L11" s="54" t="s">
         <v>103</v>
@@ -11089,17 +11157,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005B1120F001D1794FAA6F4057E3355991" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="62349bcdb43c26c508700efba1cb50b1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f20a0681-8b2f-4a46-9dab-cf1520193f81" xmlns:ns3="932fafb7-d8e0-4a14-bee3-33aad5c71309" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0e5d6db3f342a25e0e30f4a2965162e1" ns2:_="" ns3:_="">
     <xsd:import namespace="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
@@ -11288,6 +11345,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -11298,23 +11366,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1424D28F-D6A9-45ED-AED5-A0D744400EE5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11333,6 +11384,23 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
docs : màj rapport, livraison finale
</commit_message>
<xml_diff>
--- a/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
+++ b/docs/jdt/Journal-de-Travail_BorminKiril.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\px20umf\Documents\github\PlotThoseLines\docs\jdt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85DB7A06-2284-4737-B7B8-E09F3D9F734E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F330880-6A18-4B0C-9A91-F356F0AA43D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4725" yWindow="1155" windowWidth="21600" windowHeight="11745" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1650" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="118">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -292,12 +292,18 @@
     <t>Correction d'affichage pour les écrans de haute résolution</t>
   </si>
   <si>
+    <t>pour 20.10</t>
+  </si>
+  <si>
     <t>Création de logo et son utilisation dans le projet</t>
   </si>
   <si>
     <t>Ajout de légendes pour chaque axe du graphique</t>
   </si>
   <si>
+    <t>pour 25.10</t>
+  </si>
+  <si>
     <t>Analyse du feedback du chef de projet</t>
   </si>
   <si>
@@ -316,6 +322,39 @@
     <t>Déplacement de la logique de merge des séries dans une classe séparée</t>
   </si>
   <si>
+    <t>Explication des détails pour le projet par le chef de projet, et démarage de la journée</t>
+  </si>
+  <si>
+    <t>pour 26.10</t>
+  </si>
+  <si>
+    <t>Création et mise en place de projet de test</t>
+  </si>
+  <si>
+    <t>J'ai rencontré des difficultés lors d'installation des extentions pour les tests</t>
+  </si>
+  <si>
+    <t>Création des tests pour le Parser et le SeriesMerger</t>
+  </si>
+  <si>
+    <t>Disscution sur l'avancement du projet et sur certaines parties du code avec le chef de projet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mise à jour du rapport </t>
+  </si>
+  <si>
+    <t>Analyse des points restants, il faut encore finir le rapport</t>
+  </si>
+  <si>
+    <t>pour 28.10</t>
+  </si>
+  <si>
+    <t>J'ai completé les bilans dans le rapport</t>
+  </si>
+  <si>
+    <t>pour 29.10</t>
+  </si>
+  <si>
     <t>Total heures TPI</t>
   </si>
   <si>
@@ -349,37 +388,7 @@
     <t>Total</t>
   </si>
   <si>
-    <t>Explication des détails pour le projet par le chef de projet, et démarage de la journée</t>
-  </si>
-  <si>
-    <t>Création et mise en place de projet de test</t>
-  </si>
-  <si>
-    <t>J'ai rencontré des difficultés lors d'installation des extentions pour les tests</t>
-  </si>
-  <si>
-    <t>pour 20.10</t>
-  </si>
-  <si>
-    <t>pour 25.10</t>
-  </si>
-  <si>
-    <t>pour 26.10</t>
-  </si>
-  <si>
-    <t>Création des tests pour le Parser et le SeriesMerger</t>
-  </si>
-  <si>
-    <t>Disscution sur l'avancement du projet et sur certaines parties du code avec le chef de projet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mise à jour du rapport </t>
-  </si>
-  <si>
-    <t>Analyse des points restants, il faut encore finir le rapport</t>
-  </si>
-  <si>
-    <t>J'ai completé les bilans dans le rapport</t>
+    <t>Finalisation de rapport et livraison des fichiers</t>
   </si>
 </sst>
 </file>
@@ -956,7 +965,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-F5FE-49EE-BE4F-11D09FE0E927}"/>
+              <c16:uniqueId val="{00000000-70E4-44E3-9C16-24CB42CC8929}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1057,7 +1066,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-52C2-4B5A-983C-EA8938461D4F}"/>
+              <c16:uniqueId val="{00000000-860A-47B4-9A02-12967DE0E791}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1204,7 +1213,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-C531-458E-AD92-848B15585BFF}"/>
+              <c16:uniqueId val="{00000000-0068-4B7F-A845-5AD764A336A1}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1276,23 +1285,23 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.18471337579617833</c:v>
+                  <c:v>0.18124999999999999</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.75159235668789814</c:v>
+                  <c:v>0.75624999999999998</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>6.3694267515923567E-2</c:v>
+                  <c:v>6.25E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-C531-458E-AD92-848B15585BFF}"/>
+              <c16:uniqueId val="{00000001-0068-4B7F-A845-5AD764A336A1}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1669,7 +1678,7 @@
       <c r="B3" s="85"/>
       <c r="C3" s="65" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>26 heures 10 minutes</v>
+        <v>26 heures 40 minutes</v>
       </c>
       <c r="D3" s="16"/>
       <c r="E3" s="3"/>
@@ -1688,11 +1697,11 @@
       </c>
       <c r="D4" s="16">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>1090</v>
+        <v>1120</v>
       </c>
       <c r="E4" s="16">
         <f>SUM(C4:D4)</f>
-        <v>1570</v>
+        <v>1600</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -2926,7 +2935,7 @@
         <v>0 h 55 min</v>
       </c>
       <c r="I50" t="s">
-        <v>107</v>
+        <v>85</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -2945,7 +2954,7 @@
         <v>22</v>
       </c>
       <c r="F51" s="21" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G51" s="38"/>
       <c r="H51" t="str">
@@ -2969,7 +2978,7 @@
         <v>22</v>
       </c>
       <c r="F52" s="21" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G52" s="37"/>
       <c r="H52" t="str">
@@ -2977,7 +2986,7 @@
         <v>2 h 40 min</v>
       </c>
       <c r="I52" t="s">
-        <v>108</v>
+        <v>88</v>
       </c>
     </row>
     <row r="53" spans="1:9" ht="63" x14ac:dyDescent="0.25">
@@ -2996,10 +3005,10 @@
         <v>18</v>
       </c>
       <c r="F53" s="21" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="G53" s="38" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="H53" t="str">
         <f t="shared" si="0"/>
@@ -3022,7 +3031,7 @@
         <v>22</v>
       </c>
       <c r="F54" s="21" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G54" s="37"/>
       <c r="H54" t="str">
@@ -3046,7 +3055,7 @@
         <v>22</v>
       </c>
       <c r="F55" s="21" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G55" s="38"/>
       <c r="H55" t="str">
@@ -3070,7 +3079,7 @@
         <v>22</v>
       </c>
       <c r="F56" s="21" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G56" s="37"/>
       <c r="H56" t="str">
@@ -3094,7 +3103,7 @@
         <v>22</v>
       </c>
       <c r="F57" s="21" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="G57" s="38"/>
       <c r="H57" t="str">
@@ -3118,7 +3127,7 @@
         <v>18</v>
       </c>
       <c r="F58" s="37" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="G58" s="37"/>
       <c r="H58" t="str">
@@ -3126,7 +3135,7 @@
         <v>3 h 00 min</v>
       </c>
       <c r="I58" t="s">
-        <v>109</v>
+        <v>96</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -3147,10 +3156,10 @@
         <v>22</v>
       </c>
       <c r="F59" s="38" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="G59" s="38" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="H59" t="str">
         <f t="shared" si="0"/>
@@ -3173,7 +3182,7 @@
         <v>22</v>
       </c>
       <c r="F60" s="37" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="G60" s="37"/>
       <c r="H60" t="str">
@@ -3197,7 +3206,7 @@
         <v>18</v>
       </c>
       <c r="F61" s="38" t="s">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="G61" s="38"/>
       <c r="H61" t="str">
@@ -3221,7 +3230,7 @@
         <v>22</v>
       </c>
       <c r="F62" s="37" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="G62" s="37"/>
       <c r="H62" t="str">
@@ -3272,14 +3281,17 @@
         <v>32</v>
       </c>
       <c r="G64" s="37" t="s">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="H64" t="str">
         <f t="shared" si="0"/>
         <v>1 h 20 min</v>
       </c>
-    </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I64" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" s="61">
         <f>IF(ISBLANK(B65),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B65))</f>
         <v>44</v>
@@ -3297,33 +3309,44 @@
         <v>22</v>
       </c>
       <c r="F65" s="38" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="G65" s="38" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="H65" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A66" s="60" t="str">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A66" s="60">
         <f>IF(ISBLANK(B66),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B66))</f>
-        <v/>
-      </c>
-      <c r="B66" s="28"/>
+        <v>44</v>
+      </c>
+      <c r="B66" s="28">
+        <v>46324</v>
+      </c>
       <c r="C66" s="29"/>
-      <c r="D66" s="30"/>
-      <c r="E66" s="31"/>
-      <c r="F66" s="37"/>
+      <c r="D66" s="30">
+        <v>30</v>
+      </c>
+      <c r="E66" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="F66" s="37" t="s">
+        <v>117</v>
+      </c>
       <c r="G66" s="37"/>
       <c r="H66" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0 h 30 min</v>
+      </c>
+      <c r="I66" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" s="61" t="str">
         <f>IF(ISBLANK(B67),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B67))</f>
         <v/>
@@ -3339,7 +3362,7 @@
         <v/>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" s="60" t="str">
         <f>IF(ISBLANK(B68),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B68))</f>
         <v/>
@@ -3355,7 +3378,7 @@
         <v/>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" s="61" t="str">
         <f>IF(ISBLANK(B69),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B69))</f>
         <v/>
@@ -3371,7 +3394,7 @@
         <v/>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" s="60" t="str">
         <f>IF(ISBLANK(B70),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B70))</f>
         <v/>
@@ -3387,7 +3410,7 @@
         <v/>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" s="61" t="str">
         <f>IF(ISBLANK(B71),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B71))</f>
         <v/>
@@ -3403,7 +3426,7 @@
         <v/>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" s="60" t="str">
         <f>IF(ISBLANK(B72),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B72))</f>
         <v/>
@@ -3419,7 +3442,7 @@
         <v/>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" s="61" t="str">
         <f>IF(ISBLANK(B73),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B73))</f>
         <v/>
@@ -3435,7 +3458,7 @@
         <v/>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" s="60" t="str">
         <f>IF(ISBLANK(B74),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B74))</f>
         <v/>
@@ -3451,7 +3474,7 @@
         <v/>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" s="61" t="str">
         <f>IF(ISBLANK(B75),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B75))</f>
         <v/>
@@ -3467,7 +3490,7 @@
         <v/>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" s="60" t="str">
         <f>IF(ISBLANK(B76),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B76))</f>
         <v/>
@@ -3483,7 +3506,7 @@
         <v/>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" s="61" t="str">
         <f>IF(ISBLANK(B77),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B77))</f>
         <v/>
@@ -3499,7 +3522,7 @@
         <v/>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" s="60" t="str">
         <f>IF(ISBLANK(B78),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B78))</f>
         <v/>
@@ -3515,7 +3538,7 @@
         <v/>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" s="61" t="str">
         <f>IF(ISBLANK(B79),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B79))</f>
         <v/>
@@ -3531,7 +3554,7 @@
         <v/>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" s="60" t="str">
         <f>IF(ISBLANK(B80),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B80))</f>
         <v/>
@@ -10827,9 +10850,9 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.69999998807907104" right="0.69999998807907104" top="0.75" bottom="0.75" header="0.30000001192092896" footer="0.30000001192092896"/>
-  <pageSetup paperSize="9" scale="45" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="35" orientation="landscape" r:id="rId1"/>
   <rowBreaks count="1" manualBreakCount="1">
-    <brk id="50" max="16383" man="1"/>
+    <brk id="66" max="16383" man="1"/>
   </rowBreaks>
   <tableParts count="1">
     <tablePart r:id="rId2"/>
@@ -10854,13 +10877,13 @@
   <sheetData>
     <row r="2" spans="1:14" ht="21" x14ac:dyDescent="0.35">
       <c r="E2" s="64" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="F2" s="66">
         <v>90</v>
       </c>
       <c r="G2" s="64" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="L2" s="17"/>
       <c r="M2" s="42"/>
@@ -10873,42 +10896,42 @@
     </row>
     <row r="4" spans="1:14" ht="21" x14ac:dyDescent="0.35">
       <c r="E4" s="64" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="L4" s="64" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="M4" s="39"/>
       <c r="N4" s="18"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="B5" t="s">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="C5" s="39" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
       <c r="D5" s="40"/>
       <c r="E5" s="43" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="F5" s="44" t="s">
-        <v>101</v>
+        <v>114</v>
       </c>
       <c r="G5" s="45" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="L5" s="46" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="M5" s="47" t="s">
-        <v>101</v>
+        <v>114</v>
       </c>
       <c r="N5" s="48" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
@@ -10934,7 +10957,7 @@
       </c>
       <c r="G6" s="70">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.18471337579617833</v>
+        <v>0.18124999999999999</v>
       </c>
       <c r="L6" s="49" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10955,11 +10978,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>760</v>
+        <v>790</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>1180</v>
+        <v>1210</v>
       </c>
       <c r="E7" s="71" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10967,11 +10990,11 @@
       </c>
       <c r="F7" s="72" t="str">
         <f t="shared" si="1"/>
-        <v>19 h 40 min</v>
+        <v>20 h 10 min</v>
       </c>
       <c r="G7" s="73">
         <f>SUM(A7:B7)/$C$11</f>
-        <v>0.75159235668789814</v>
+        <v>0.75624999999999998</v>
       </c>
       <c r="L7" s="51" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11045,7 +11068,7 @@
       </c>
       <c r="G9" s="73">
         <f>SUM(A9:B9)/$C$11</f>
-        <v>6.3694267515923567E-2</v>
+        <v>6.25E-2</v>
       </c>
       <c r="L9" s="53" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11101,25 +11124,25 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>1090</v>
+        <v>1120</v>
       </c>
       <c r="C11">
         <f t="shared" si="0"/>
-        <v>1570</v>
+        <v>1600</v>
       </c>
       <c r="E11" s="79" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="F11" s="69" t="str">
         <f t="shared" si="1"/>
-        <v>26 h 10 min</v>
+        <v>26 h 40 min</v>
       </c>
       <c r="G11" s="80">
         <f>C11/C12</f>
-        <v>0.29074074074074074</v>
+        <v>0.29629629629629628</v>
       </c>
       <c r="L11" s="54" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="M11" s="55"/>
       <c r="N11" s="58">
@@ -11157,6 +11180,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005B1120F001D1794FAA6F4057E3355991" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="62349bcdb43c26c508700efba1cb50b1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f20a0681-8b2f-4a46-9dab-cf1520193f81" xmlns:ns3="932fafb7-d8e0-4a14-bee3-33aad5c71309" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0e5d6db3f342a25e0e30f4a2965162e1" ns2:_="" ns3:_="">
     <xsd:import namespace="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
@@ -11345,27 +11388,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1424D28F-D6A9-45ED-AED5-A0D744400EE5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11382,29 +11430,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>